<commit_message>
Исправлен apm_m_driver. Добавлены тесты: 1) rw_with_wait_states_test 2) full_session_test
</commit_message>
<xml_diff>
--- a/testplan/testplan.xlsx
+++ b/testplan/testplan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SV\apb_protocol_UVM_tb\testplan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2FA687C-62D9-4B77-94DE-CE94112FDEBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{237987E0-FB21-497F-9E51-D26E61EB68CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="38">
   <si>
     <t>Директория</t>
   </si>
@@ -58,9 +58,6 @@
   </si>
   <si>
     <t>README.md</t>
-  </si>
-  <si>
-    <t>-</t>
   </si>
   <si>
     <t>single_write_slave2_test</t>
@@ -155,9 +152,6 @@
   <si>
     <t>1) Сброс
 2) Подавать случайные операции со случайными задержками</t>
-  </si>
-  <si>
-    <t>В разработке</t>
   </si>
   <si>
     <t>back_to_back_write_test</t>
@@ -651,13 +645,13 @@
         <v>10</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="75" x14ac:dyDescent="0.25">
@@ -665,22 +659,22 @@
         <v>7</v>
       </c>
       <c r="B3" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="12" t="s">
         <v>12</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>13</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="112.5" x14ac:dyDescent="0.25">
@@ -688,22 +682,22 @@
         <v>7</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="112.5" x14ac:dyDescent="0.25">
@@ -711,22 +705,22 @@
         <v>7</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="112.5" x14ac:dyDescent="0.25">
@@ -734,22 +728,22 @@
         <v>7</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="112.5" x14ac:dyDescent="0.25">
@@ -757,22 +751,22 @@
         <v>7</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="112.5" x14ac:dyDescent="0.25">
@@ -780,22 +774,22 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="56.25" x14ac:dyDescent="0.25">
@@ -803,22 +797,22 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="G9" s="2" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="56.25" x14ac:dyDescent="0.25">
@@ -826,22 +820,22 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="18.75" x14ac:dyDescent="0.25">

</xml_diff>